<commit_message>
arreglo generacion de modulos excel
- nueva hoja base oculta
- nombres de tablas por periodo
- correccion al duplicar tablas excel
- limpieza de tablas heredadas
- mejoras generales en generar_modulo.py
</commit_message>
<xml_diff>
--- a/templates/Modulo-00.xlsx
+++ b/templates/Modulo-00.xlsx
@@ -54,13 +54,13 @@
     <t>C.C.T.</t>
   </si>
   <si>
-    <t>ANEXO DE RELEVAMIENTO DE DATOS</t>
-  </si>
-  <si>
     <t>C.U.I.T</t>
   </si>
   <si>
     <t>ACTA N°</t>
+  </si>
+  <si>
+    <t>ANEXO RELEVAMIENTO DE DATOS</t>
   </si>
 </sst>
 </file>
@@ -247,9 +247,6 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -262,6 +259,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -931,7 +931,7 @@
   <sheetData>
     <row r="1" spans="2:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B1" s="16" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H1" s="22"/>
       <c r="I1" s="23"/>
@@ -956,33 +956,33 @@
       <c r="D4" s="18"/>
       <c r="E4" s="17"/>
       <c r="F4" s="17"/>
-      <c r="H4" s="25"/>
-      <c r="I4" s="25"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
     </row>
     <row r="5" spans="2:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="26" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="27"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="29"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="26" t="s">
+      <c r="B5" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="26"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="25" t="s">
         <v>10</v>
       </c>
       <c r="I5" s="19"/>
     </row>
     <row r="6" spans="2:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="30"/>
-      <c r="D6" s="28"/>
-      <c r="E6" s="28"/>
-      <c r="F6" s="29"/>
-      <c r="G6" s="28"/>
-      <c r="H6" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="29"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="25" t="s">
         <v>9</v>
       </c>
       <c r="I6" s="19"/>

</xml_diff>

<commit_message>
Se Agregaron lo Modulos deU.P.F.P.A.R.A., Con sus columnas especificas que no dependen de la base de datos, se cargo un diagrama para aclarar como es la distribucion del flujo
</commit_message>
<xml_diff>
--- a/templates/Modulo-00.xlsx
+++ b/templates/Modulo-00.xlsx
@@ -138,7 +138,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -175,11 +175,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -262,33 +277,130 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="19">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
+  <dxfs count="20">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -304,15 +416,20 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
         <color theme="1"/>
         <name val="Arial"/>
         <scheme val="none"/>
@@ -323,6 +440,47 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -346,11 +504,16 @@
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
         <color theme="1"/>
         <name val="Arial"/>
         <scheme val="none"/>
@@ -382,11 +545,16 @@
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
         <color theme="1"/>
         <name val="Arial"/>
         <scheme val="none"/>
@@ -397,6 +565,47 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -420,11 +629,16 @@
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
         <color theme="1"/>
         <name val="Arial"/>
         <scheme val="none"/>
@@ -465,12 +679,6 @@
         <name val="Arial"/>
         <scheme val="none"/>
       </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -489,129 +697,6 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -627,7 +712,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Modulo_00_000" displayName="Modulo_00_000" ref="B9:I21" totalsRowCount="1" headerRowDxfId="18" dataDxfId="17" totalsRowDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Modulo_00_0000" displayName="Modulo_00_0000" ref="B9:I21" totalsRowCount="1" headerRowDxfId="0" dataDxfId="19" totalsRowDxfId="18" headerRowBorderDxfId="1">
   <autoFilter ref="B9:I20">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -639,14 +724,14 @@
     <filterColumn colId="7" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="8">
-    <tableColumn id="1" name="Legajo" totalsRowLabel="Total" dataDxfId="15" totalsRowDxfId="14"/>
-    <tableColumn id="2" name="Apellido y Nombre" dataDxfId="13" totalsRowDxfId="12"/>
-    <tableColumn id="3" name="C.U.I.L" dataDxfId="11" totalsRowDxfId="10"/>
-    <tableColumn id="4" name="Fecha de Ingreso" dataDxfId="9" totalsRowDxfId="8"/>
-    <tableColumn id="5" name="Convenio" dataDxfId="7" totalsRowDxfId="6"/>
-    <tableColumn id="6" name="Afiliado" dataDxfId="5" totalsRowDxfId="4"/>
-    <tableColumn id="7" name="Categoria" dataDxfId="3" totalsRowDxfId="2"/>
-    <tableColumn id="8" name="Remuneracion Bruta" totalsRowFunction="count" dataDxfId="1" totalsRowDxfId="0"/>
+    <tableColumn id="1" name="Legajo" totalsRowLabel="Total" dataDxfId="17" totalsRowDxfId="16"/>
+    <tableColumn id="2" name="Apellido y Nombre" dataDxfId="15" totalsRowDxfId="14"/>
+    <tableColumn id="3" name="C.U.I.L" dataDxfId="13" totalsRowDxfId="12"/>
+    <tableColumn id="4" name="Fecha de Ingreso" dataDxfId="11" totalsRowDxfId="10"/>
+    <tableColumn id="5" name="Convenio" dataDxfId="9" totalsRowDxfId="8"/>
+    <tableColumn id="6" name="Afiliado" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="7" name="Categoria" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="8" name="Remuneracion Bruta" totalsRowFunction="count" dataDxfId="3" totalsRowDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -924,8 +1009,8 @@
     <col min="5" max="5" width="14.7109375" style="2" customWidth="1"/>
     <col min="6" max="6" width="11" style="1" customWidth="1"/>
     <col min="7" max="7" width="10.7109375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="22.7109375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="20.85546875" style="3" customWidth="1"/>
+    <col min="8" max="8" width="24.7109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.7109375" style="3" customWidth="1"/>
     <col min="10" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
@@ -1002,28 +1087,28 @@
       <c r="I8" s="8"/>
     </row>
     <row r="9" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="E9" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="H9" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="I9" s="12" t="s">
+      <c r="I9" s="32" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1137,7 +1222,7 @@
       <c r="H20" s="11"/>
       <c r="I20" s="12"/>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="13" t="s">
         <v>8</v>
       </c>
@@ -1147,8 +1232,8 @@
       <c r="F21" s="11"/>
       <c r="G21" s="13"/>
       <c r="H21" s="11"/>
-      <c r="I21" s="12">
-        <f>SUBTOTAL(103,Modulo_00_000[Remuneracion Bruta])</f>
+      <c r="I21" s="15">
+        <f>SUBTOTAL(103,Modulo_00_0000[Remuneracion Bruta])</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>